<commit_message>
feat: manager approval workflow + admin notifications
- Fixed url_for('dashboard') bug -> employee_dashboard
- Added Status column backfill for all legacy Excel files
- get_pending_requests() now treats None status as Pending
- Manager dashboard shows all pending leave/WFH/HD requests
- Approved requests logged to approved_log.json
- Admin dashboard shows only Approved requests as notifications
- Added .gitignore for pycache and temp files
</commit_message>
<xml_diff>
--- a/2026/January/07-jan-2026.xlsx
+++ b/2026/January/07-jan-2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="07-jan-2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-jan-2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -481,6 +481,16 @@
           <t>Timestamp</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Action By</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -511,6 +521,12 @@
           <t>2026-01-21 14:29:22</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>